<commit_message>
Add AGENTS.md for project guidance; update .gitignore to include AGENTS.md and clean up unused imports in various files
</commit_message>
<xml_diff>
--- a/Datasheets/pcbuilder_import_data_20260902_cpuseries.xlsx
+++ b/Datasheets/pcbuilder_import_data_20260902_cpuseries.xlsx
@@ -1,15 +1,415 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="CpuSeries" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CpuSeries" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -36,12 +436,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4e3bea87-6932-4819-8db2-85728f581277</t>
+          <t>7fd65649-5c4a-49b6-bb70-e34d4f4a8908</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>320f15bb-4f9f-4727-9a17-028865d1ac1c</t>
+          <t>5e6269d3-c539-4ecc-a46a-8d8074c64997</t>
         </is>
       </c>
     </row>
@@ -53,12 +453,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4e3bea87-6932-4819-8db2-85728f581277</t>
+          <t>7fd65649-5c4a-49b6-bb70-e34d4f4a8908</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>320f15bb-4f9f-4727-9a17-028865d1ac1c</t>
+          <t>5e6269d3-c539-4ecc-a46a-8d8074c64997</t>
         </is>
       </c>
     </row>
@@ -70,12 +470,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4e3bea87-6932-4819-8db2-85728f581277</t>
+          <t>7fd65649-5c4a-49b6-bb70-e34d4f4a8908</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>a2c9596d-60f1-4ee9-a3d0-063cb9249d23</t>
+          <t>5a06a35f-634a-45ae-92c1-d7a6b25481f5</t>
         </is>
       </c>
     </row>
@@ -87,12 +487,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4e3bea87-6932-4819-8db2-85728f581277</t>
+          <t>7fd65649-5c4a-49b6-bb70-e34d4f4a8908</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>a2c9596d-60f1-4ee9-a3d0-063cb9249d23</t>
+          <t>5a06a35f-634a-45ae-92c1-d7a6b25481f5</t>
         </is>
       </c>
     </row>
@@ -104,12 +504,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4e3bea87-6932-4819-8db2-85728f581277</t>
+          <t>7fd65649-5c4a-49b6-bb70-e34d4f4a8908</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>a2c9596d-60f1-4ee9-a3d0-063cb9249d23</t>
+          <t>5a06a35f-634a-45ae-92c1-d7a6b25481f5</t>
         </is>
       </c>
     </row>
@@ -121,12 +521,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4e3bea87-6932-4819-8db2-85728f581277</t>
+          <t>7fd65649-5c4a-49b6-bb70-e34d4f4a8908</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>89f39647-02c6-4e3a-a7e2-11537ac4b025</t>
+          <t>5490f478-840a-4da1-bd54-f97256622ee3</t>
         </is>
       </c>
     </row>
@@ -138,12 +538,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04bd0d18-b83d-4e30-a5d2-c052ab3c84ca</t>
+          <t>dd191e11-e1e5-4b65-89c0-a28a4d8f6ce1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>906cdde8-5cc2-4022-ac34-8cbc677e4872</t>
+          <t>77c2dbd0-a223-4c80-aea2-3a39e80043de</t>
         </is>
       </c>
     </row>
@@ -155,12 +555,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04bd0d18-b83d-4e30-a5d2-c052ab3c84ca</t>
+          <t>dd191e11-e1e5-4b65-89c0-a28a4d8f6ce1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2ff24ca3-bc12-421e-9912-0e44bd2748c7</t>
+          <t>7494de81-7d22-40c3-9b29-46f56e4b3cdd</t>
         </is>
       </c>
     </row>
@@ -172,12 +572,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04bd0d18-b83d-4e30-a5d2-c052ab3c84ca</t>
+          <t>dd191e11-e1e5-4b65-89c0-a28a4d8f6ce1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2ff24ca3-bc12-421e-9912-0e44bd2748c7</t>
+          <t>7494de81-7d22-40c3-9b29-46f56e4b3cdd</t>
         </is>
       </c>
     </row>
@@ -189,15 +589,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>04bd0d18-b83d-4e30-a5d2-c052ab3c84ca</t>
+          <t>dd191e11-e1e5-4b65-89c0-a28a4d8f6ce1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2ff24ca3-bc12-421e-9912-0e44bd2748c7</t>
+          <t>7494de81-7d22-40c3-9b29-46f56e4b3cdd</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>